<commit_message>
Quote bank trimmed to 129 for Year 8 suitability
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gu1VzQkkrTnot1kzm8PSSu
</commit_message>
<xml_diff>
--- a/data/Agorian_Quote_Bank.xlsx
+++ b/data/Agorian_Quote_Bank.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <strike val="1"/>
+      <color rgb="00999999"/>
     </font>
   </fonts>
   <fills count="3">
@@ -54,10 +58,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1339,31 +1346,39 @@
       <c r="G33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>He who fears he will suffer already suffers what he fears.</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Michel de Montaigne, Essays</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Calm under pressure</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1393,31 +1408,39 @@
       <c r="G35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Although the world is full of suffering, it is full also of the overcoming of it.</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Helen Keller, Optimism</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Calm under pressure</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1609,31 +1632,39 @@
       <c r="G43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Before enlightenment, chop wood, carry water. After enlightenment, chop wood, carry water.</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Zen saying</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Calm under pressure</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>Proverb or saying</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1690,31 +1721,39 @@
       <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Keep calm and carry on.</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>British Ministry of Information poster, 1939</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Calm under pressure</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -1771,31 +1810,39 @@
       <c r="G49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Reading maketh a full man, conference a ready man, and writing an exact man.</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Francis Bacon, Of Studies</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Value of learning</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -1960,31 +2007,39 @@
       <c r="G56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Not having heard something is not as good as having heard it. Having heard it is not as good as having seen it. Having seen it is not as good as knowing it. Knowing it is not as good as putting it into practice.</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Xunzi</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Value of learning</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2365,31 +2420,39 @@
       <c r="G71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="3" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Teach thy tongue to say I do not know, and thou shalt progress.</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>Maimonides</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>Value of learning</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -2554,31 +2617,39 @@
       <c r="G78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="3" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>We must form our minds by reading deep rather than wide.</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>Quintilian, Institutio Oratoria</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Value of learning</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3040,31 +3111,39 @@
       <c r="G96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="B97" s="2" t="inlineStr">
+      <c r="B97" s="3" t="inlineStr">
         <is>
           <t>The desire for safety stands against every great and noble enterprise.</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C97" s="3" t="inlineStr">
         <is>
           <t>Tacitus, Annals</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>Courage</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -3256,31 +3335,39 @@
       <c r="G104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="3" t="n">
         <v>104</v>
       </c>
-      <c r="B105" s="2" t="inlineStr">
+      <c r="B105" s="3" t="inlineStr">
         <is>
           <t>No man ever steps in the same river twice.</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr">
+      <c r="C105" s="3" t="inlineStr">
         <is>
           <t>Heraclitus</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
+      <c r="D105" s="3" t="inlineStr">
         <is>
           <t>Thinking</t>
         </is>
       </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr"/>
-      <c r="G105" s="2" t="inlineStr"/>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -3445,31 +3532,39 @@
       <c r="G111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="3" t="n">
         <v>111</v>
       </c>
-      <c r="B112" s="2" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>He who has a why to live can bear almost any how.</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C112" s="3" t="inlineStr">
         <is>
           <t>Friedrich Nietzsche, Twilight of the Idols</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D112" s="3" t="inlineStr">
         <is>
           <t>Thinking</t>
         </is>
       </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="2" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -3526,31 +3621,39 @@
       <c r="G114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="3" t="n">
         <v>114</v>
       </c>
-      <c r="B115" s="2" t="inlineStr">
+      <c r="B115" s="3" t="inlineStr">
         <is>
           <t>Become who you are, having learned what that is.</t>
         </is>
       </c>
-      <c r="C115" s="2" t="inlineStr">
+      <c r="C115" s="3" t="inlineStr">
         <is>
           <t>Pindar, Pythian Odes</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
+      <c r="D115" s="3" t="inlineStr">
         <is>
           <t>Thinking</t>
         </is>
       </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F115" s="2" t="inlineStr"/>
-      <c r="G115" s="2" t="inlineStr"/>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -4093,31 +4196,39 @@
       <c r="G135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="3" t="n">
         <v>135</v>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B136" s="3" t="inlineStr">
         <is>
           <t>It is not that we have a short time to live, but that we waste a lot of it.</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
+      <c r="C136" s="3" t="inlineStr">
         <is>
           <t>Seneca, On the Shortness of Life</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="D136" s="3" t="inlineStr">
         <is>
           <t>Effort and practice</t>
         </is>
       </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>In the named work</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr"/>
-      <c r="G136" s="2" t="inlineStr"/>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>In the named work</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>Cut on review (heavy, abstract or archaic for Year 8)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">

</xml_diff>